<commit_message>
feat: improve visual audit and examples
</commit_message>
<xml_diff>
--- a/examples/templates/branddocs_template.xlsx
+++ b/examples/templates/branddocs_template.xlsx
@@ -11,10 +11,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="client_name">'Cover'!$B$4</definedName>
+    <definedName name="dashboard_kpis">'Dashboard'!$A$4:$H$5</definedName>
     <definedName name="data_block">'Data'!$A$2:$D$4</definedName>
     <definedName name="headline_kpi">'Summary'!$B$9</definedName>
     <definedName name="inputs_block">'Inputs'!$A$4:$C$7</definedName>
@@ -22,8 +25,11 @@
     <definedName name="period">'Cover'!$B$5</definedName>
     <definedName name="report_subtitle">'Cover'!$A$2</definedName>
     <definedName name="report_title">'Cover'!$A$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Cover'!$A$1:$E$9</definedName>
+    <definedName name="scenario_block">'Scenarios'!$A$5:$D$8</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Cover'!$A$1:$G$13</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Model'!$A$1:$G$27</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Dashboard'!$A$1:$H$24</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Scenarios'!$A$1:$D$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -31,13 +37,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="_($* #,##0.00_);_($* (#,##0.00);_($* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="_($* #,##0_);_($* (#,##0);_($* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="0.00x"/>
+    <numFmt numFmtId="168" formatCode="_($* #,##0_);_($* (#,##0);_($* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,6 +78,12 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="20"/>
     </font>
     <font>
@@ -84,6 +97,18 @@
       <b val="1"/>
       <color rgb="FF16213F"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF16213F"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FF2B7CD3"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -128,7 +153,7 @@
       </bottom>
     </border>
   </borders>
-  <cellStyleXfs count="6">
+  <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -139,36 +164,64 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="2"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="2"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2"/>
-  </cellStyleXfs>
-  <cellXfs count="14">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  </cellStyleXfs>
+  <cellXfs count="24">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="5"/>
     <xf numFmtId="3" fontId="3" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="5"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="3"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="4"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="5"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
     <cellStyle name="BrandDocsTitle" xfId="1" hidden="0"/>
     <cellStyle name="BrandDocsHeader" xfId="2" hidden="0"/>
     <cellStyle name="BrandDocsCurrency" xfId="3" hidden="0"/>
     <cellStyle name="BrandDocsPercent" xfId="4" hidden="0"/>
     <cellStyle name="BrandDocsInput" xfId="5" hidden="0"/>
+    <cellStyle name="BrandDocsKPI" xfId="6" hidden="0"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -431,16 +484,113 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Net revenue</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!B7</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="2B7CD3"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$8:$A$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$B$8:$B$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>BrandDocs</author>
+  </authors>
+  <commentList>
+    <comment ref="B3" authorId="0" shapeId="0">
+      <text>
+        <t>Synthetic scenario selector used by formulas and visual QA.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>7</row>
+      <row>8</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="609600" cy="609600"/>
+    <ext cx="1714500" cy="428625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -515,6 +665,33 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3060000" cy="2160000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BrandDocsDataTbl" displayName="BrandDocsDataTbl" ref="A3:G7" headerRowCount="1">
   <autoFilter ref="A3:G7"/>
@@ -528,6 +705,19 @@
     <tableColumn id="7" name="% of FY"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BrandDocsScenarioTbl" displayName="BrandDocsScenarioTbl" ref="A5:D8" headerRowCount="1">
+  <autoFilter ref="A5:D8"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Scenario"/>
+    <tableColumn id="2" name="Revenue multiplier"/>
+    <tableColumn id="3" name="Margin delta"/>
+    <tableColumn id="4" name="Narrative"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
@@ -820,11 +1010,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -841,7 +1036,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
           <t>Prepared for</t>
@@ -852,8 +1047,28 @@
           <t>BrandDocs Corp (synthetic demo)</t>
         </is>
       </c>
-    </row>
-    <row r="5">
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>FY net revenue</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Net margin</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Brand audit</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
           <t>Reporting period</t>
@@ -862,6 +1077,24 @@
       <c r="B5" t="inlineStr">
         <is>
           <t>FY2025 (Q1-Q4)</t>
+        </is>
+      </c>
+      <c r="D5" s="4">
+        <f>Summary!B4</f>
+        <v/>
+      </c>
+      <c r="E5" s="5">
+        <f>Summary!B8</f>
+        <v/>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Deep QA</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>3 formats</t>
         </is>
       </c>
     </row>
@@ -871,24 +1104,26 @@
           <t>Generated on</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>2026-01-15</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="4" t="n"/>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="9" t="n"/>
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="1" fitToWidth="1"/>
@@ -910,84 +1145,84 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Model Inputs</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Units sold</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="12" t="n">
         <v>29070</v>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Unit price</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Discount rate</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="14" t="n">
         <v>0.12</v>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>pct</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Tax rate</t>
         </is>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="14" t="n">
         <v>0.22</v>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>pct</t>
         </is>
@@ -1017,44 +1252,44 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Revenue Model</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Line item</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>FY Total</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>% of FY</t>
         </is>
@@ -1066,23 +1301,23 @@
           <t>Gross revenue</t>
         </is>
       </c>
-      <c r="B4" s="11" t="n">
+      <c r="B4" s="15" t="n">
         <v>320000</v>
       </c>
-      <c r="C4" s="11" t="n">
+      <c r="C4" s="15" t="n">
         <v>351000</v>
       </c>
-      <c r="D4" s="11" t="n">
+      <c r="D4" s="15" t="n">
         <v>372500</v>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="E4" s="15" t="n">
         <v>410000</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="15">
         <f>SUM(B4:E4)</f>
         <v/>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="16">
         <f>IF($F$7=0,0,F4/$F$7)</f>
         <v/>
       </c>
@@ -1093,23 +1328,23 @@
           <t>Discounts</t>
         </is>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="15" t="n">
         <v>-38400</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="15" t="n">
         <v>-42120</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="15" t="n">
         <v>-44700</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="15" t="n">
         <v>-49200</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="15">
         <f>SUM(B5:E5)</f>
         <v/>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="16">
         <f>IF($F$7=0,0,F5/$F$7)</f>
         <v/>
       </c>
@@ -1120,23 +1355,23 @@
           <t>Returns</t>
         </is>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="15" t="n">
         <v>-9600</v>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C6" s="15" t="n">
         <v>-10530</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="15" t="n">
         <v>-11175</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="15" t="n">
         <v>-12300</v>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="15">
         <f>SUM(B6:E6)</f>
         <v/>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="16">
         <f>IF($F$7=0,0,F6/$F$7)</f>
         <v/>
       </c>
@@ -1147,27 +1382,27 @@
           <t>Net revenue</t>
         </is>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="15">
         <f>SUM(B4:B6)</f>
         <v/>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="15">
         <f>SUM(C4:C6)</f>
         <v/>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="15">
         <f>SUM(D4:D6)</f>
         <v/>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="15">
         <f>SUM(E4:E6)</f>
         <v/>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="15">
         <f>SUM(B7:E7)</f>
         <v/>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="16">
         <f>IF($F$7=0,0,F7/$F$7)</f>
         <v/>
       </c>
@@ -1178,7 +1413,7 @@
           <t>Subtotal (visible)</t>
         </is>
       </c>
-      <c r="F9" s="11">
+      <c r="F9" s="15">
         <f>SUBTOTAL(9,F4:F6)</f>
         <v/>
       </c>
@@ -1229,19 +1464,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Executive Summary</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -1253,7 +1488,7 @@
           <t>FY net revenue</t>
         </is>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="15">
         <f>Model!F7</f>
         <v/>
       </c>
@@ -1264,7 +1499,7 @@
           <t>Units sold (input)</t>
         </is>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="15">
         <f>Inputs!B4</f>
         <v/>
       </c>
@@ -1275,7 +1510,7 @@
           <t>Unit price (input)</t>
         </is>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="13">
         <f>Inputs!B5</f>
         <v/>
       </c>
@@ -1286,7 +1521,7 @@
           <t>Implied gross</t>
         </is>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="13">
         <f>Inputs!B4*Inputs!B5</f>
         <v/>
       </c>
@@ -1297,7 +1532,7 @@
           <t>Net margin</t>
         </is>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="14">
         <f>IF(B7=0,0,B4/B7)</f>
         <v/>
       </c>
@@ -1322,6 +1557,332 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Executive Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Formula-backed snapshot generated from the model, inputs, and summary tabs</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>FY net revenue</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Net margin</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Input units</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19">
+        <f>Summary!B4</f>
+        <v/>
+      </c>
+      <c r="C5" s="20">
+        <f>Summary!B8</f>
+        <v/>
+      </c>
+      <c r="E5" s="19">
+        <f>Summary!B5</f>
+        <v/>
+      </c>
+      <c r="G5" s="21">
+        <f>Scenarios!B3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Quarter</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Net revenue</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="B8" s="15">
+        <f>Model!B7</f>
+        <v/>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="B9" s="15">
+        <f>Model!C7</f>
+        <v/>
+      </c>
+      <c r="C9" s="16">
+        <f>IF(B8=0,0,B9/B8-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B10" s="15">
+        <f>Model!D7</f>
+        <v/>
+      </c>
+      <c r="C10" s="16">
+        <f>IF(B9=0,0,B10/B9-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="B11" s="15">
+        <f>Model!E7</f>
+        <v/>
+      </c>
+      <c r="C11" s="16">
+        <f>IF(B10=0,0,B11/B10-1)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="C4:D4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B8:B11">
+    <cfRule type="dataBar" priority="1">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="002B7CD3"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Scenario Controls</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Selected scenario</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Revenue multiplier</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Margin delta</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Narrative</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Plan case</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Upside</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Faster adoption</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Downside</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Cost pressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Scenario revenue</t>
+        </is>
+      </c>
+      <c r="B10" s="15">
+        <f>Summary!B4*INDEX(B6:B8,MATCH($B$3,A6:A8,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Scenario margin</t>
+        </is>
+      </c>
+      <c r="B11" s="16">
+        <f>Summary!B8+INDEX(C6:C8,MATCH($B$3,A6:A8,0))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Base,Upside,Downside"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="1" fitToWidth="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1337,29 +1898,29 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>2025-10-01</t>
         </is>
@@ -1374,12 +1935,12 @@
           <t>Widget</t>
         </is>
       </c>
-      <c r="D2" s="13" t="n">
+      <c r="D2" s="23" t="n">
         <v>12500</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>2025-10-02</t>
         </is>
@@ -1394,12 +1955,12 @@
           <t>Gadget</t>
         </is>
       </c>
-      <c r="D3" s="13" t="n">
+      <c r="D3" s="23" t="n">
         <v>9800</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>2025-10-03</t>
         </is>
@@ -1414,7 +1975,7 @@
           <t>Widget</t>
         </is>
       </c>
-      <c r="D4" s="13" t="n">
+      <c r="D4" s="23" t="n">
         <v>14200</v>
       </c>
     </row>
@@ -1424,7 +1985,7 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="15">
         <f>SUM(D2:D4)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
feat(examples): broaden the xlsx showcase CF + number-format coverage
Add the two remaining common conditional-formatting families to the Model sheet -
an icon set (3 traffic lights on the %-of-FY column) and a top-N rule (top 3 of the
quarter grid) - so the CF inventory the comprehension model reads now spans
colorScale/cellIs/expression/dataBar/iconSet/top10. Also give the negative line
items (Discounts/Returns) a red-negative accounting mask on existing cells (no
named-region geometry change), surfacing a distinct number-format the inventory
aggregates (7 -> 8 masks). Rebuilt template extracts with 0 problems; the example
determinism guard and kitchen-sink stay green.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/templates/branddocs_template.xlsx
+++ b/examples/templates/branddocs_template.xlsx
@@ -37,12 +37,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="_($* #,##0.00_);_($* (#,##0.00);_($* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="0.00x"/>
-    <numFmt numFmtId="168" formatCode="_($* #,##0_);_($* (#,##0);_($* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="#,##0;[Red](#,##0)"/>
+    <numFmt numFmtId="168" formatCode="0.00x"/>
+    <numFmt numFmtId="169" formatCode="_($* #,##0_);_($* (#,##0);_($* &quot;-&quot;_);_(@_)"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -168,7 +169,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
@@ -206,6 +207,7 @@
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="3"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="4"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -219,8 +221,8 @@
     <xf numFmtId="49" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="5"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="3" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="5"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -231,7 +233,14 @@
     <cellStyle name="BrandDocsInput" xfId="5" hidden="0"/>
     <cellStyle name="BrandDocsKPI" xfId="6" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF63BE7B"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1345,19 +1354,19 @@
           <t>Discounts</t>
         </is>
       </c>
-      <c r="B5" s="15" t="n">
+      <c r="B5" s="17" t="n">
         <v>-38400</v>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C5" s="17" t="n">
         <v>-42120</v>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="D5" s="17" t="n">
         <v>-44700</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="17" t="n">
         <v>-49200</v>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="17">
         <f>SUM(B5:E5)</f>
         <v/>
       </c>
@@ -1372,19 +1381,19 @@
           <t>Returns</t>
         </is>
       </c>
-      <c r="B6" s="15" t="n">
+      <c r="B6" s="17" t="n">
         <v>-9600</v>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="17" t="n">
         <v>-10530</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="17" t="n">
         <v>-11175</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="17" t="n">
         <v>-12300</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="17">
         <f>SUM(B6:E6)</f>
         <v/>
       </c>
@@ -1447,15 +1456,25 @@
         <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
+    <cfRule type="top10" rank="3" priority="5" dxfId="0"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G4:G7">
-    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="1">
       <formula>0.5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F4:F6">
-    <cfRule type="expression" priority="3" dxfId="1">
+    <cfRule type="expression" priority="3" dxfId="2">
       <formula>F4&lt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4:G6">
+    <cfRule type="iconSet" priority="4">
+      <iconSet iconSet="3TrafficLights1">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="percent" val="33"/>
+        <cfvo type="percent" val="67"/>
+      </iconSet>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1527,7 +1546,7 @@
           <t>Unit price (input)</t>
         </is>
       </c>
-      <c r="B6" s="17">
+      <c r="B6" s="18">
         <f>Inputs!B5</f>
         <v/>
       </c>
@@ -1538,7 +1557,7 @@
           <t>Implied gross</t>
         </is>
       </c>
-      <c r="B7" s="17">
+      <c r="B7" s="18">
         <f>Inputs!B4*Inputs!B5</f>
         <v/>
       </c>
@@ -1549,7 +1568,7 @@
           <t>Net margin</t>
         </is>
       </c>
-      <c r="B8" s="18">
+      <c r="B8" s="19">
         <f>IF(B7=0,0,B4/B7)</f>
         <v/>
       </c>
@@ -1593,14 +1612,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Executive Dashboard</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>Formula-backed snapshot generated from the model, inputs, and summary tabs</t>
         </is>
@@ -1629,19 +1648,19 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21">
+      <c r="A5" s="22">
         <f>Summary!B4</f>
         <v/>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="23">
         <f>Summary!B8</f>
         <v/>
       </c>
-      <c r="E5" s="21">
+      <c r="E5" s="22">
         <f>Summary!B5</f>
         <v/>
       </c>
-      <c r="G5" s="23">
+      <c r="G5" s="24">
         <f>Scenarios!B3</f>
         <v/>
       </c>
@@ -1814,10 +1833,10 @@
           <t>Base</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n">
+      <c r="B6" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="18" t="n">
+      <c r="C6" s="19" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -1832,10 +1851,10 @@
           <t>Upside</t>
         </is>
       </c>
-      <c r="B7" s="24" t="n">
+      <c r="B7" s="25" t="n">
         <v>1.12</v>
       </c>
-      <c r="C7" s="18" t="n">
+      <c r="C7" s="19" t="n">
         <v>0.025</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -1850,10 +1869,10 @@
           <t>Downside</t>
         </is>
       </c>
-      <c r="B8" s="24" t="n">
+      <c r="B8" s="25" t="n">
         <v>0.91</v>
       </c>
-      <c r="C8" s="18" t="n">
+      <c r="C8" s="19" t="n">
         <v>-0.035</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -1952,7 +1971,7 @@
           <t>Widget</t>
         </is>
       </c>
-      <c r="D2" s="25" t="n">
+      <c r="D2" s="26" t="n">
         <v>12500</v>
       </c>
     </row>
@@ -1972,7 +1991,7 @@
           <t>Gadget</t>
         </is>
       </c>
-      <c r="D3" s="25" t="n">
+      <c r="D3" s="26" t="n">
         <v>9800</v>
       </c>
     </row>
@@ -1992,7 +2011,7 @@
           <t>Widget</t>
         </is>
       </c>
-      <c r="D4" s="25" t="n">
+      <c r="D4" s="26" t="n">
         <v>14200</v>
       </c>
     </row>

</xml_diff>